<commit_message>
fix : tableau de synthese
</commit_message>
<xml_diff>
--- a/assets/docs/Dimitri-Tableau de synthese.xlsx
+++ b/assets/docs/Dimitri-Tableau de synthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\portfolio\assets\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B9814F-7464-4513-9F54-67DED9FCCCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41974B48-2EF3-465D-BEB0-6CC7C99D994F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -118,9 +118,6 @@
   <si>
     <t xml:space="preserve">Réalisation en cours de formation
 </t>
-  </si>
-  <si>
-    <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
     <r>
@@ -193,6 +190,18 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>19/01/2026 au 27/02/2026</t>
+  </si>
+  <si>
+    <t>Développement : Participer à la création de formulaires de maintenance dans le cadre d’un ERP Développement : Participer à la création de workflows opérationnels dans le cadre d’un ERP Développement : Participer à la modification et à l’ajout de nouvelles fonctionnalités aux applications existantes
+Tests / QA : Tester et s’assurer que les modules ou modifications développés répondent aux exigences et aux résultats attendus
+Tests / QA : Tester les modifications réalisées par les coéquipiers afin de s’assurer que les exigences sont respectées
+Solution IA : Créer et entraîner un modèle d’intelligence artificielle basé sur les besoins du client et les objectifs du projet</t>
+  </si>
+  <si>
+    <t>Réalisations en milieu professionnel en cours de seconde année : FRCI</t>
   </si>
 </sst>
 </file>
@@ -774,15 +783,39 @@
     <xf numFmtId="16" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -823,30 +856,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1169,56 +1178,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="30"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" s="46"/>
-      <c r="H3" s="52"/>
+      <c r="A3" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="30"/>
+      <c r="H3" s="36"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="48" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="50"/>
+      <c r="A4" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34"/>
       <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
@@ -1226,26 +1235,26 @@
         <v>4</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
+      <c r="A5" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="52"/>
     </row>
     <row r="6" spans="1:43" ht="77.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="48" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1268,8 +1277,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="221.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="41"/>
+      <c r="A7" s="38"/>
+      <c r="B7" s="49"/>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
@@ -1325,16 +1334,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="41"/>
       <c r="I8" s="21"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1373,24 +1382,24 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="203" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" s="22"/>
       <c r="D9" s="22"/>
       <c r="E9" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1430,24 +1439,24 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="223" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="22"/>
       <c r="E10" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I10"/>
       <c r="J10"/>
@@ -1487,14 +1496,14 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="281" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -1537,16 +1546,16 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="36"/>
+      <c r="A12" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="44"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1585,22 +1594,24 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="228.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="22"/>
+        <v>23</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>33</v>
+      </c>
       <c r="D13" s="22"/>
       <c r="E13" s="22"/>
       <c r="F13" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H13" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I13"/>
       <c r="J13"/>
@@ -1639,16 +1650,16 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A14" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="39"/>
+      <c r="A14" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="46"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1685,15 +1696,25 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="8"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="352" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>34</v>
+      </c>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
+      <c r="E15" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>33</v>
+      </c>
       <c r="G15" s="14"/>
-      <c r="H15" s="15"/>
+      <c r="H15" s="22" t="s">
+        <v>33</v>
+      </c>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -2093,11 +2114,6 @@
     <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2105,6 +2121,11 @@
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2115,21 +2136,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010021F7977E49F44542ABC169D3385720BE" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2cf713f46d33035be00877ff8f959ac0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3e941104-c427-4bbd-984f-032c9c413468" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4c16e54e4b70d5728734523a24a24c88" ns2:_="">
     <xsd:import namespace="3e941104-c427-4bbd-984f-032c9c413468"/>
@@ -2267,31 +2273,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E2624D4-D0F5-4CDD-8F7C-B158102636B5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="3e941104-c427-4bbd-984f-032c9c413468"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76564368-5BF8-48E2-AA91-E85E538DFFE3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AD92159-81FB-4C72-AE74-77C4F4A0B31E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2307,4 +2304,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76564368-5BF8-48E2-AA91-E85E538DFFE3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E2624D4-D0F5-4CDD-8F7C-B158102636B5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="3e941104-c427-4bbd-984f-032c9c413468"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>